<commit_message>
Subjects Json List Updated
</commit_message>
<xml_diff>
--- a/RESULTS/2017/CLASS/JSS1/FIRST/Mathematics/results.xlsx
+++ b/RESULTS/2017/CLASS/JSS1/FIRST/Mathematics/results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -475,6 +475,21 @@
       <c r="L1" t="inlineStr">
         <is>
           <t>Submitted At</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Session</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Submission Status</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Termination Reason</t>
         </is>
       </c>
     </row>

</xml_diff>